<commit_message>
added qwen thinking and medgemma results
</commit_message>
<xml_diff>
--- a/control/results/Anatomy-vs-Image_Left-Right-Questions.xlsx
+++ b/control/results/Anatomy-vs-Image_Left-Right-Questions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\archlinux\home\omarg\VLMs-Medical-Imaging\control\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F2C626C-37D4-4360-981A-DD9242996E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA3991E5-55EF-44AC-B88F-561107452C60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Anatomy_Accuracy_Mean</t>
   </si>
@@ -67,7 +67,13 @@
     <t>Model Name</t>
   </si>
   <si>
-    <t>Qwen 3.5</t>
+    <t>Qwen 3.5 9B (Instruct)</t>
+  </si>
+  <si>
+    <t>Qwen 3.5 9B (Thinking 1024)</t>
+  </si>
+  <si>
+    <t>MedGemma 1.5 (Instruct)</t>
   </si>
 </sst>
 </file>
@@ -119,13 +125,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -431,66 +448,65 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" customWidth="1"/>
+    <col min="1" max="1" width="25.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.44140625" customWidth="1"/>
     <col min="3" max="3" width="21.6640625" customWidth="1"/>
     <col min="4" max="4" width="18.44140625" customWidth="1"/>
-    <col min="5" max="5" width="16.33203125" customWidth="1"/>
-    <col min="6" max="11" width="0" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="21" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="22.6640625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="21.5546875" customWidth="1"/>
-    <col min="13" max="13" width="19.21875" customWidth="1"/>
-    <col min="14" max="14" width="17.21875" customWidth="1"/>
-    <col min="15" max="15" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="15" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="L1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="M1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="N1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="O1" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
@@ -510,34 +526,126 @@
         <v>7.7997406072178232E-3</v>
       </c>
       <c r="F2" s="1">
+        <v>0.51938319642599795</v>
+      </c>
+      <c r="G2" s="1">
+        <v>4.8642135269456209E-3</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0.56211873962124337</v>
+      </c>
+      <c r="I2" s="1">
+        <v>8.0943205165412372E-3</v>
+      </c>
+      <c r="J2" s="4">
         <v>1242</v>
       </c>
-      <c r="G2" s="1">
+      <c r="K2" s="4">
         <v>1217</v>
       </c>
-      <c r="H2" s="1">
+      <c r="L2" s="4">
         <v>1224</v>
       </c>
-      <c r="I2" s="1">
+      <c r="M2" s="4">
         <v>1064</v>
       </c>
-      <c r="J2" s="1">
+      <c r="N2" s="4">
         <v>1089</v>
       </c>
-      <c r="K2" s="1">
+      <c r="O2" s="4">
         <v>1082</v>
       </c>
-      <c r="L2" s="1">
-        <v>0.51938319642599795</v>
-      </c>
-      <c r="M2" s="1">
-        <v>4.8642135269456209E-3</v>
-      </c>
-      <c r="N2" s="1">
-        <v>0.56211873962124337</v>
-      </c>
-      <c r="O2" s="1">
-        <v>8.0943205165412372E-3</v>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="3">
+        <v>0.49233882625036141</v>
+      </c>
+      <c r="C3" s="3">
+        <v>8.0702658873708193E-3</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0.34939440165509161</v>
+      </c>
+      <c r="E3" s="3">
+        <v>9.7628160585980957E-3</v>
+      </c>
+      <c r="F3" s="3">
+        <v>0.44920017293558151</v>
+      </c>
+      <c r="G3" s="3">
+        <v>6.4850843060959562E-4</v>
+      </c>
+      <c r="H3" s="3">
+        <v>0.24733112716504571</v>
+      </c>
+      <c r="I3" s="3">
+        <v>3.692719279268709E-3</v>
+      </c>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5">
+        <v>1118</v>
+      </c>
+      <c r="L3" s="5">
+        <v>1155</v>
+      </c>
+      <c r="M3" s="5">
+        <v>1133</v>
+      </c>
+      <c r="N3" s="5">
+        <v>1188</v>
+      </c>
+      <c r="O3" s="5">
+        <v>1151</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="3">
+        <v>0.53469210754553342</v>
+      </c>
+      <c r="C4" s="3">
+        <v>5.2038161318300191E-3</v>
+      </c>
+      <c r="D4" s="3">
+        <v>0.47064214433585028</v>
+      </c>
+      <c r="E4" s="3">
+        <v>6.1802937750250796E-3</v>
+      </c>
+      <c r="F4" s="3">
+        <v>0.50439544602968722</v>
+      </c>
+      <c r="G4" s="3">
+        <v>7.7500098917704019E-3</v>
+      </c>
+      <c r="H4" s="3">
+        <v>0.4190652535932885</v>
+      </c>
+      <c r="I4" s="3">
+        <v>1.0852107933010511E-2</v>
+      </c>
+      <c r="J4" s="3">
+        <v>1233</v>
+      </c>
+      <c r="K4" s="6">
+        <v>1245</v>
+      </c>
+      <c r="L4" s="6">
+        <v>1221</v>
+      </c>
+      <c r="M4" s="6">
+        <v>1073</v>
+      </c>
+      <c r="N4" s="6">
+        <v>1061</v>
+      </c>
+      <c r="O4" s="6">
+        <v>1085</v>
       </c>
     </row>
   </sheetData>

</xml_diff>